<commit_message>
feat(auth): implement authentication foundation
</commit_message>
<xml_diff>
--- a/FAIR_CRM_PROJECT.xlsx
+++ b/FAIR_CRM_PROJECT.xlsx
@@ -1064,7 +1064,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" style="41" min="1" max="1"/>
@@ -1249,6 +1249,23 @@
       <c r="E10" t="inlineStr">
         <is>
           <t>v0.2.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>POST /auth/login with seeded admin credentials</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Done</t>
         </is>
       </c>
     </row>
@@ -1972,9 +1989,21 @@
       <c r="D11" s="58" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="58" t="n"/>
-      <c r="B12" s="58" t="n"/>
-      <c r="C12" s="58" t="n"/>
+      <c r="A12" s="58" t="inlineStr">
+        <is>
+          <t>v0.2.2</t>
+        </is>
+      </c>
+      <c r="B12" s="58" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C12" s="58" t="inlineStr">
+        <is>
+          <t>Authentication foundation: JWT from env, auth service, POST /auth/login, GET /auth/me, dependencies.</t>
+        </is>
+      </c>
       <c r="D12" s="58" t="n"/>
     </row>
     <row r="13">
@@ -2374,7 +2403,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="41" min="1" max="1"/>
@@ -2600,6 +2629,28 @@
       <c r="D10" t="inlineStr">
         <is>
           <t>v0.2.1</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Authentication foundation: login, JWT, /auth/me, auth service layer</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>v0.2.2</t>
         </is>
       </c>
     </row>
@@ -11188,7 +11239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="41" min="1" max="1"/>
@@ -12275,6 +12326,40 @@
       <c r="E40" s="58" t="inlineStr">
         <is>
           <t>Done</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>POST /auth/login</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Email/password login, returns bearer token</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>GET /auth/me</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Auth</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Return current authenticated user</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(api): add repository layer and API foundation
</commit_message>
<xml_diff>
--- a/FAIR_CRM_PROJECT.xlsx
+++ b/FAIR_CRM_PROJECT.xlsx
@@ -1621,10 +1621,26 @@
       <c r="D14" s="58" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="58" t="n"/>
-      <c r="B15" s="58" t="n"/>
-      <c r="C15" s="58" t="n"/>
-      <c r="D15" s="58" t="n"/>
+      <c r="A15" s="58" t="inlineStr">
+        <is>
+          <t>Architecture</t>
+        </is>
+      </c>
+      <c r="B15" s="58" t="inlineStr">
+        <is>
+          <t>Router -&gt; Service -&gt; Repository -&gt; Database</t>
+        </is>
+      </c>
+      <c r="C15" s="58" t="inlineStr">
+        <is>
+          <t>Accepted</t>
+        </is>
+      </c>
+      <c r="D15" s="58" t="inlineStr">
+        <is>
+          <t>v0.2.3</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="58" t="n"/>
@@ -2007,9 +2023,21 @@
       <c r="D12" s="58" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="58" t="n"/>
-      <c r="B13" s="58" t="n"/>
-      <c r="C13" s="58" t="n"/>
+      <c r="A13" s="58" t="inlineStr">
+        <is>
+          <t>v0.2.3</t>
+        </is>
+      </c>
+      <c r="B13" s="58" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="C13" s="58" t="inlineStr">
+        <is>
+          <t>Repository layer, centralized exceptions, API response foundation, logging, auth service refactor.</t>
+        </is>
+      </c>
       <c r="D13" s="58" t="n"/>
     </row>
     <row r="14">
@@ -2403,7 +2431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" style="41" min="1" max="1"/>
@@ -2651,6 +2679,28 @@
       <c r="D11" t="inlineStr">
         <is>
           <t>v0.2.2</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Repository layer and API foundation (BaseRepository, UserRepository, exceptions, logging)</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Done</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>v0.2.3</t>
         </is>
       </c>
     </row>

</xml_diff>